<commit_message>
Update AXON data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/AXON_data.xlsx
+++ b/data/AXON_data.xlsx
@@ -11049,7 +11049,7 @@
         <v>213.08676</v>
       </c>
       <c r="L2" t="n">
-        <v>48.835297</v>
+        <v>48.76833</v>
       </c>
       <c r="M2" t="n">
         <v>2.42</v>
@@ -11129,7 +11129,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:09:09</t>
+          <t>2026-09-08 08:53:01</t>
         </is>
       </c>
     </row>

</xml_diff>